<commit_message>
Update Oct 2026 Trapezoidal Flume Calibration Final.xlsx
</commit_message>
<xml_diff>
--- a/data/New Data Oct 2026/Oct 2026 Trapezoidal Flume Calibration Final.xlsx
+++ b/data/New Data Oct 2026/Oct 2026 Trapezoidal Flume Calibration Final.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30602"/>
-  <workbookPr codeName="ThisWorkbook"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://colostate-my.sharepoint.com/personal/bschaub_colostate_edu/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c7d62234183fd3ba/Documents/GitHub/3d-flume-uncertainty-analysis/data/New Data Oct 2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{AB680839-0861-48A1-B7A0-D9FEA9FDC587}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{43C32F17-1129-416A-A178-F9A048A89AEB}"/>
+    <workbookView xWindow="-38520" yWindow="-30" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{43C32F17-1129-416A-A178-F9A048A89AEB}"/>
   </bookViews>
   <sheets>
     <sheet name="Base Calibration (6-point)" sheetId="6" r:id="rId1"/>
@@ -135,7 +135,7 @@
     <numFmt numFmtId="165" formatCode="0.00000"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -715,7 +715,7 @@
             <c:strRef>
               <c:f>'Base Calibration (6-point)'!$B$7:$F$7</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>3D Printed Flume #2</c:v>
                 </c:pt>
@@ -810,7 +810,7 @@
             <c:strRef>
               <c:f>'Base Calibration (6-point)'!$H$7:$L$7</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>Fiberglass Flume</c:v>
                 </c:pt>
@@ -1475,7 +1475,7 @@
             <c:strRef>
               <c:f>'Base Calibration (6-point)'!$B$7:$F$7</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>3D Printed Flume #2</c:v>
                 </c:pt>
@@ -1570,7 +1570,7 @@
             <c:strRef>
               <c:f>'Base Calibration (6-point)'!$H$7:$L$7</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>Fiberglass Flume</c:v>
                 </c:pt>
@@ -2141,7 +2141,7 @@
             <c:strRef>
               <c:f>'Detailed Calibration (10-point)'!$B$7:$F$7</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>3D Printed Flume #1 </c:v>
                 </c:pt>
@@ -2260,7 +2260,7 @@
             <c:strRef>
               <c:f>'Detailed Calibration (10-point)'!$H$7:$L$7</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>3D Printed Flume #2 </c:v>
                 </c:pt>
@@ -2379,7 +2379,7 @@
             <c:strRef>
               <c:f>'Detailed Calibration (10-point)'!$N$7:$R$7</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>Fiberglass Flume</c:v>
                 </c:pt>
@@ -3191,7 +3191,7 @@
             <c:strRef>
               <c:f>'Detailed Calibration (10-point)'!$H$7:$L$7</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>3D Printed Flume #2 </c:v>
                 </c:pt>
@@ -3310,7 +3310,7 @@
             <c:strRef>
               <c:f>'Detailed Calibration (10-point)'!$N$7:$R$7</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>Fiberglass Flume</c:v>
                 </c:pt>
@@ -3908,7 +3908,7 @@
             <c:strRef>
               <c:f>'Detailed Calibration (10-point)'!$B$7:$F$7</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>3D Printed Flume #1 </c:v>
                 </c:pt>
@@ -4016,7 +4016,7 @@
             <c:strRef>
               <c:f>'Detailed Calibration (10-point)'!$H$7:$L$7</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>3D Printed Flume #2 </c:v>
                 </c:pt>
@@ -4124,7 +4124,7 @@
             <c:strRef>
               <c:f>'Detailed Calibration (10-point)'!$N$7:$R$7</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>Fiberglass Flume</c:v>
                 </c:pt>
@@ -4572,7 +4572,7 @@
             <c:strRef>
               <c:f>'Detailed Calibration (10-point)'!$B$7:$F$7</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>3D Printed Flume #1 </c:v>
                 </c:pt>
@@ -4680,7 +4680,7 @@
             <c:strRef>
               <c:f>'Detailed Calibration (10-point)'!$H$7:$L$7</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>3D Printed Flume #2 </c:v>
                 </c:pt>
@@ -4788,7 +4788,7 @@
             <c:strRef>
               <c:f>'Detailed Calibration (10-point)'!$N$7:$R$7</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>Fiberglass Flume</c:v>
                 </c:pt>
@@ -9073,7 +9073,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD719889-40B6-4341-ADB8-A84703AE80DA}">
   <dimension ref="B1:O51"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.5703125" customWidth="1"/>
@@ -9087,14 +9087,14 @@
     <col min="17" max="17" width="10.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="15.75" thickBot="1"/>
-    <row r="2" spans="2:12" ht="15.75" thickBot="1">
+    <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="61" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="62"/>
     </row>
-    <row r="3" spans="2:12">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="17" t="s">
         <v>1</v>
       </c>
@@ -9103,7 +9103,7 @@
         <v>0.125</v>
       </c>
     </row>
-    <row r="4" spans="2:12">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="19" t="s">
         <v>2</v>
       </c>
@@ -9112,7 +9112,7 @@
         <v>1.0416666666666666E-2</v>
       </c>
     </row>
-    <row r="5" spans="2:12" ht="15.75" thickBot="1">
+    <row r="5" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="20" t="s">
         <v>3</v>
       </c>
@@ -9120,8 +9120,8 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="6" spans="2:12" ht="15.75" thickBot="1"/>
-    <row r="7" spans="2:12" ht="15.75" thickBot="1">
+    <row r="6" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="58" t="s">
         <v>4</v>
       </c>
@@ -9137,7 +9137,7 @@
       <c r="K7" s="59"/>
       <c r="L7" s="60"/>
     </row>
-    <row r="8" spans="2:12" ht="15.75" thickBot="1">
+    <row r="8" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="8" t="s">
         <v>6</v>
       </c>
@@ -9157,7 +9157,7 @@
       <c r="K8" s="28"/>
       <c r="L8" s="29"/>
     </row>
-    <row r="9" spans="2:12" ht="41.25" customHeight="1" thickBot="1">
+    <row r="9" spans="2:12" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="9" t="s">
         <v>7</v>
       </c>
@@ -9189,7 +9189,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="2:12">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="12">
         <v>0.1</v>
       </c>
@@ -9227,7 +9227,7 @@
         <v>8.6167650209522208E-4</v>
       </c>
     </row>
-    <row r="11" spans="2:12">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="12">
         <v>0.15</v>
       </c>
@@ -9265,7 +9265,7 @@
         <v>1.4882148393177306E-4</v>
       </c>
     </row>
-    <row r="12" spans="2:12">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="12">
         <v>0.2</v>
       </c>
@@ -9303,7 +9303,7 @@
         <v>1.3991598173513672E-3</v>
       </c>
     </row>
-    <row r="13" spans="2:12">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="12">
         <v>0.25</v>
       </c>
@@ -9341,7 +9341,7 @@
         <v>3.3968330506695273E-4</v>
       </c>
     </row>
-    <row r="14" spans="2:12">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="12">
         <v>0.3</v>
       </c>
@@ -9379,7 +9379,7 @@
         <v>2.1376369964920482E-4</v>
       </c>
     </row>
-    <row r="15" spans="2:12" ht="15.75" thickBot="1">
+    <row r="15" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="16">
         <v>0.32</v>
       </c>
@@ -9417,7 +9417,7 @@
         <v>9.1220073475006011E-5</v>
       </c>
     </row>
-    <row r="16" spans="2:12" ht="15.75" thickBot="1">
+    <row r="16" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
@@ -9439,7 +9439,7 @@
         <v>2.2562228323644237E-2</v>
       </c>
     </row>
-    <row r="17" spans="2:15" ht="15.75" thickBot="1">
+    <row r="17" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E17" s="20" t="s">
         <v>13</v>
       </c>
@@ -9455,19 +9455,19 @@
         <v>3.0543248815695259E-3</v>
       </c>
     </row>
-    <row r="18" spans="2:15" ht="15.75" thickBot="1">
+    <row r="18" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="65" t="s">
         <v>14</v>
       </c>
       <c r="C18" s="66"/>
     </row>
-    <row r="19" spans="2:15" ht="15.75" thickBot="1">
+    <row r="19" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="63" t="s">
         <v>15</v>
       </c>
       <c r="C19" s="64"/>
     </row>
-    <row r="20" spans="2:15" ht="15.75" thickBot="1">
+    <row r="20" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="17" t="s">
         <v>16</v>
       </c>
@@ -9475,7 +9475,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="2:15">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B21" s="21">
         <v>0</v>
       </c>
@@ -9486,7 +9486,7 @@
       <c r="N21" s="1"/>
       <c r="O21" s="1"/>
     </row>
-    <row r="22" spans="2:15">
+    <row r="22" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B22" s="22">
         <v>0.02</v>
       </c>
@@ -9500,7 +9500,7 @@
       <c r="N22" s="1"/>
       <c r="O22" s="1"/>
     </row>
-    <row r="23" spans="2:15" ht="15" customHeight="1">
+    <row r="23" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="22">
         <v>0.04</v>
       </c>
@@ -9514,7 +9514,7 @@
       <c r="N23" s="1"/>
       <c r="O23" s="1"/>
     </row>
-    <row r="24" spans="2:15">
+    <row r="24" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B24" s="22">
         <v>0.06</v>
       </c>
@@ -9528,7 +9528,7 @@
       <c r="N24" s="1"/>
       <c r="O24" s="1"/>
     </row>
-    <row r="25" spans="2:15">
+    <row r="25" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B25" s="22">
         <v>0.08</v>
       </c>
@@ -9542,7 +9542,7 @@
       <c r="N25" s="1"/>
       <c r="O25" s="1"/>
     </row>
-    <row r="26" spans="2:15">
+    <row r="26" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B26" s="22">
         <v>0.1</v>
       </c>
@@ -9556,7 +9556,7 @@
       <c r="N26" s="1"/>
       <c r="O26" s="1"/>
     </row>
-    <row r="27" spans="2:15">
+    <row r="27" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B27" s="22">
         <v>0.12</v>
       </c>
@@ -9568,7 +9568,7 @@
       <c r="I27" s="3"/>
       <c r="J27" s="1"/>
     </row>
-    <row r="28" spans="2:15">
+    <row r="28" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B28" s="22">
         <v>0.14000000000000001</v>
       </c>
@@ -9580,7 +9580,7 @@
       <c r="I28" s="3"/>
       <c r="J28" s="1"/>
     </row>
-    <row r="29" spans="2:15">
+    <row r="29" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B29" s="22">
         <v>0.16</v>
       </c>
@@ -9592,7 +9592,7 @@
       <c r="I29" s="3"/>
       <c r="J29" s="1"/>
     </row>
-    <row r="30" spans="2:15">
+    <row r="30" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B30" s="22">
         <v>0.18</v>
       </c>
@@ -9601,7 +9601,7 @@
         <v>1.8575254011746728E-2</v>
       </c>
     </row>
-    <row r="31" spans="2:15">
+    <row r="31" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B31" s="22">
         <v>0.2</v>
       </c>
@@ -9610,7 +9610,7 @@
         <v>2.4377495614638721E-2</v>
       </c>
     </row>
-    <row r="32" spans="2:15">
+    <row r="32" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B32" s="22">
         <v>0.22</v>
       </c>
@@ -9619,7 +9619,7 @@
         <v>3.1173259491050275E-2</v>
       </c>
     </row>
-    <row r="33" spans="2:3">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33" s="22">
         <v>0.24</v>
       </c>
@@ -9628,7 +9628,7 @@
         <v>3.9019050934588635E-2</v>
       </c>
     </row>
-    <row r="34" spans="2:3">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B34" s="22">
         <v>0.26</v>
       </c>
@@ -9637,7 +9637,7 @@
         <v>4.7969250841353041E-2</v>
       </c>
     </row>
-    <row r="35" spans="2:3">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B35" s="22">
         <v>0.28000000000000003</v>
       </c>
@@ -9646,7 +9646,7 @@
         <v>5.8076364061848774E-2</v>
       </c>
     </row>
-    <row r="36" spans="2:3">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B36" s="22">
         <v>0.3</v>
       </c>
@@ -9655,7 +9655,7 @@
         <v>6.9391221957620625E-2</v>
       </c>
     </row>
-    <row r="37" spans="2:3">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B37" s="22">
         <v>0.32</v>
       </c>
@@ -9664,7 +9664,7 @@
         <v>8.1963150268266852E-2</v>
       </c>
     </row>
-    <row r="38" spans="2:3">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B38" s="22">
         <v>0.34</v>
       </c>
@@ -9673,7 +9673,7 @@
         <v>9.5840110140021362E-2</v>
       </c>
     </row>
-    <row r="39" spans="2:3">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B39" s="22">
         <v>0.36</v>
       </c>
@@ -9682,7 +9682,7 @@
         <v>0.11106881801065087</v>
       </c>
     </row>
-    <row r="40" spans="2:3">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B40" s="22">
         <v>0.38</v>
       </c>
@@ -9691,7 +9691,7 @@
         <v>0.12769484857347996</v>
       </c>
     </row>
-    <row r="41" spans="2:3">
+    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B41" s="22">
         <v>0.4</v>
       </c>
@@ -9700,7 +9700,7 @@
         <v>0.14576272401257673</v>
       </c>
     </row>
-    <row r="42" spans="2:3">
+    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B42" s="22">
         <v>0.42</v>
       </c>
@@ -9709,7 +9709,7 @@
         <v>0.16531599196298566</v>
       </c>
     </row>
-    <row r="43" spans="2:3">
+    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B43" s="22">
         <v>0.44</v>
       </c>
@@ -9718,7 +9718,7 @@
         <v>0.18639729411079389</v>
       </c>
     </row>
-    <row r="44" spans="2:3">
+    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B44" s="22">
         <v>0.46</v>
       </c>
@@ -9727,7 +9727,7 @@
         <v>0.20904842694716996</v>
       </c>
     </row>
-    <row r="45" spans="2:3">
+    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B45" s="22">
         <v>0.48</v>
       </c>
@@ -9736,7 +9736,7 @@
         <v>0.23331039588807301</v>
       </c>
     </row>
-    <row r="46" spans="2:3">
+    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B46" s="22">
         <v>0.5</v>
       </c>
@@ -9745,7 +9745,7 @@
         <v>0.25922346373980926</v>
       </c>
     </row>
-    <row r="47" spans="2:3">
+    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B47" s="22">
         <v>0.52</v>
       </c>
@@ -9754,7 +9754,7 @@
         <v>0.28682719431110998</v>
       </c>
     </row>
-    <row r="48" spans="2:3">
+    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B48" s="22">
         <v>0.54</v>
       </c>
@@ -9763,7 +9763,7 @@
         <v>0.31616049183163297</v>
       </c>
     </row>
-    <row r="49" spans="2:3">
+    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B49" s="22">
         <v>0.56000000000000005</v>
       </c>
@@ -9772,7 +9772,7 @@
         <v>0.34726163672521515</v>
       </c>
     </row>
-    <row r="50" spans="2:3">
+    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B50" s="22">
         <v>0.57999999999999996</v>
       </c>
@@ -9781,7 +9781,7 @@
         <v>0.38016831819691932</v>
       </c>
     </row>
-    <row r="51" spans="2:3" ht="15.75" thickBot="1">
+    <row r="51" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B51" s="23">
         <v>0.6</v>
       </c>
@@ -9806,7 +9806,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC98C4DB-F457-455A-8D27-EF7CF7D8F585}">
   <dimension ref="B1:AB55"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.5703125" customWidth="1"/>
@@ -9822,14 +9822,14 @@
     <col min="29" max="29" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:28" ht="15.75" thickBot="1"/>
-    <row r="2" spans="2:28" ht="15.75" thickBot="1">
+    <row r="1" spans="2:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="61" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="62"/>
     </row>
-    <row r="3" spans="2:28">
+    <row r="3" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B3" s="17" t="s">
         <v>18</v>
       </c>
@@ -9837,7 +9837,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="4" spans="2:28">
+    <row r="4" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B4" s="19" t="s">
         <v>2</v>
       </c>
@@ -9846,7 +9846,7 @@
         <v>3.2808398950131233E-4</v>
       </c>
     </row>
-    <row r="5" spans="2:28" ht="15.75" thickBot="1">
+    <row r="5" spans="2:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="20" t="s">
         <v>3</v>
       </c>
@@ -9854,8 +9854,8 @@
         <v>5.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="6" spans="2:28" ht="15.75" thickBot="1"/>
-    <row r="7" spans="2:28" ht="15.75" thickBot="1">
+    <row r="6" spans="2:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="2:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="58" t="s">
         <v>19</v>
       </c>
@@ -9878,7 +9878,7 @@
       <c r="Q7" s="59"/>
       <c r="R7" s="60"/>
     </row>
-    <row r="8" spans="2:28" ht="15.75" customHeight="1" thickBot="1">
+    <row r="8" spans="2:28" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="8" t="s">
         <v>21</v>
       </c>
@@ -9919,7 +9919,7 @@
       <c r="AA8" s="56"/>
       <c r="AB8" s="57"/>
     </row>
-    <row r="9" spans="2:28" ht="36" customHeight="1" thickBot="1">
+    <row r="9" spans="2:28" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="9" t="s">
         <v>7</v>
       </c>
@@ -9990,7 +9990,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="2:28" ht="36" customHeight="1">
+    <row r="10" spans="2:28" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="11">
         <v>0.02</v>
       </c>
@@ -10049,34 +10049,34 @@
         <v>0.02</v>
       </c>
       <c r="U10" s="46">
-        <f>(E10-C10)/C10</f>
+        <f t="shared" ref="U10:U19" si="7">(E10-C10)/C10</f>
         <v>0.11055496930364248</v>
       </c>
       <c r="V10" s="49">
-        <f>(K10-I10)/I10</f>
+        <f t="shared" ref="V10:V19" si="8">(K10-I10)/I10</f>
         <v>4.5019827574400616E-2</v>
       </c>
       <c r="W10" s="49">
-        <f>(Q10-O10)/O10</f>
+        <f t="shared" ref="W10:W19" si="9">(Q10-O10)/O10</f>
         <v>0.15306425042531352</v>
       </c>
       <c r="Y10" s="42">
         <v>0.02</v>
       </c>
       <c r="Z10" s="11">
-        <f>(E10-C10)*12</f>
+        <f t="shared" ref="Z10:Z19" si="10">(E10-C10)*12</f>
         <v>0.24573783786042347</v>
       </c>
       <c r="AA10" s="52">
-        <f>(K10-I10)*12</f>
+        <f t="shared" ref="AA10:AA19" si="11">(K10-I10)*12</f>
         <v>0.10006854652184127</v>
       </c>
       <c r="AB10" s="52">
-        <f>(Q10-O10)*12</f>
+        <f t="shared" ref="AB10:AB19" si="12">(Q10-O10)*12</f>
         <v>0.34022602683680259</v>
       </c>
     </row>
-    <row r="11" spans="2:28">
+    <row r="11" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B11" s="12">
         <v>0.04</v>
       </c>
@@ -10106,7 +10106,7 @@
         <v>18.79</v>
       </c>
       <c r="K11" s="14">
-        <f t="shared" ref="K11:K19" si="7">CONVERT((J11-$I$8)/100,"m","ft")</f>
+        <f t="shared" ref="K11:K19" si="13">CONVERT((J11-$I$8)/100,"m","ft")</f>
         <v>0.25065616797900253</v>
       </c>
       <c r="L11" s="36">
@@ -10124,7 +10124,7 @@
         <v>17.45</v>
       </c>
       <c r="Q11" s="14">
-        <f t="shared" ref="Q11:Q19" si="8">CONVERT((P11-$O$8)/100,"m","ft")</f>
+        <f t="shared" ref="Q11:Q19" si="14">CONVERT((P11-$O$8)/100,"m","ft")</f>
         <v>0.24606299212598426</v>
       </c>
       <c r="R11" s="36">
@@ -10135,34 +10135,34 @@
         <v>0.04</v>
       </c>
       <c r="U11" s="47">
-        <f>(E11-C11)/C11</f>
+        <f t="shared" si="7"/>
         <v>3.7105639068204611E-2</v>
       </c>
       <c r="V11" s="50">
-        <f>(K11-I11)/I11</f>
+        <f t="shared" si="8"/>
         <v>3.439779144661631E-2</v>
       </c>
       <c r="W11" s="50">
-        <f>(Q11-O11)/O11</f>
+        <f t="shared" si="9"/>
         <v>1.544285809550071E-2</v>
       </c>
       <c r="Y11" s="43">
         <v>0.04</v>
       </c>
       <c r="Z11" s="12">
-        <f>(E11-C11)*12</f>
+        <f t="shared" si="10"/>
         <v>0.10789764683748126</v>
       </c>
       <c r="AA11" s="53">
-        <f>(K11-I11)*12</f>
+        <f t="shared" si="11"/>
         <v>0.10002363108944889</v>
       </c>
       <c r="AB11" s="53">
-        <f>(Q11-O11)*12</f>
+        <f t="shared" si="12"/>
         <v>4.490552085322963E-2</v>
       </c>
     </row>
-    <row r="12" spans="2:28">
+    <row r="12" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B12" s="12">
         <v>0.06</v>
       </c>
@@ -10192,7 +10192,7 @@
         <v>19.77</v>
       </c>
       <c r="K12" s="14">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>0.28280839895013121</v>
       </c>
       <c r="L12" s="36">
@@ -10210,7 +10210,7 @@
         <v>18.84</v>
       </c>
       <c r="Q12" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>0.29166666666666669</v>
       </c>
       <c r="R12" s="36">
@@ -10221,34 +10221,34 @@
         <v>0.06</v>
       </c>
       <c r="U12" s="47">
-        <f>(E12-C12)/C12</f>
+        <f t="shared" si="7"/>
         <v>3.6692149289711234E-2</v>
       </c>
       <c r="V12" s="50">
-        <f>(K12-I12)/I12</f>
+        <f t="shared" si="8"/>
         <v>-2.6466153038718051E-3</v>
       </c>
       <c r="W12" s="50">
-        <f>(Q12-O12)/O12</f>
+        <f t="shared" si="9"/>
         <v>2.8592991873385255E-2</v>
       </c>
       <c r="Y12" s="43">
         <v>0.06</v>
       </c>
       <c r="Z12" s="12">
-        <f>(E12-C12)*12</f>
+        <f t="shared" si="10"/>
         <v>0.12485261277163895</v>
       </c>
       <c r="AA12" s="53">
-        <f>(K12-I12)*12</f>
+        <f t="shared" si="11"/>
         <v>-9.0056549448973566E-3</v>
       </c>
       <c r="AB12" s="53">
-        <f>(Q12-O12)*12</f>
+        <f t="shared" si="12"/>
         <v>9.7293557653528318E-2</v>
       </c>
     </row>
-    <row r="13" spans="2:28">
+    <row r="13" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B13" s="12">
         <v>0.08</v>
       </c>
@@ -10278,7 +10278,7 @@
         <v>21.13</v>
       </c>
       <c r="K13" s="14">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>0.32742782152230965</v>
       </c>
       <c r="L13" s="36">
@@ -10296,7 +10296,7 @@
         <v>20.05</v>
       </c>
       <c r="Q13" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>0.33136482939632556</v>
       </c>
       <c r="R13" s="36">
@@ -10307,34 +10307,34 @@
         <v>0.08</v>
       </c>
       <c r="U13" s="47">
-        <f>(E13-C13)/C13</f>
+        <f t="shared" si="7"/>
         <v>2.7697219772907095E-2</v>
       </c>
       <c r="V13" s="50">
-        <f>(K13-I13)/I13</f>
+        <f t="shared" si="8"/>
         <v>3.2871928835207606E-2</v>
       </c>
       <c r="W13" s="50">
-        <f>(Q13-O13)/O13</f>
+        <f t="shared" si="9"/>
         <v>4.5291230584729648E-2</v>
       </c>
       <c r="Y13" s="43">
         <v>0.08</v>
       </c>
       <c r="Z13" s="12">
-        <f>(E13-C13)*12</f>
+        <f t="shared" si="10"/>
         <v>0.10536261171541073</v>
       </c>
       <c r="AA13" s="53">
-        <f>(K13-I13)*12</f>
+        <f t="shared" si="11"/>
         <v>0.12504765108548899</v>
       </c>
       <c r="AB13" s="53">
-        <f>(Q13-O13)*12</f>
+        <f t="shared" si="12"/>
         <v>0.17229174557367988</v>
       </c>
     </row>
-    <row r="14" spans="2:28">
+    <row r="14" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B14" s="12">
         <v>0.1</v>
       </c>
@@ -10364,7 +10364,7 @@
         <v>21.69</v>
       </c>
       <c r="K14" s="14">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>0.34580052493438324</v>
       </c>
       <c r="L14" s="36">
@@ -10382,7 +10382,7 @@
         <v>20.69</v>
       </c>
       <c r="Q14" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>0.35236220472440954</v>
       </c>
       <c r="R14" s="36">
@@ -10393,34 +10393,34 @@
         <v>0.1</v>
       </c>
       <c r="U14" s="47">
-        <f>(E14-C14)/C14</f>
+        <f t="shared" si="7"/>
         <v>1.8482648660047223E-2</v>
       </c>
       <c r="V14" s="50">
-        <f>(K14-I14)/I14</f>
+        <f t="shared" si="8"/>
         <v>4.4800716466886713E-4</v>
       </c>
       <c r="W14" s="50">
-        <f>(Q14-O14)/O14</f>
+        <f t="shared" si="9"/>
         <v>1.9431840317698814E-2</v>
       </c>
       <c r="Y14" s="43">
         <v>0.1</v>
       </c>
       <c r="Z14" s="12">
-        <f>(E14-C14)*12</f>
+        <f t="shared" si="10"/>
         <v>7.6661370462644651E-2</v>
       </c>
       <c r="AA14" s="53">
-        <f>(K14-I14)*12</f>
+        <f t="shared" si="11"/>
         <v>1.8582208563451275E-3</v>
       </c>
       <c r="AB14" s="53">
-        <f>(Q14-O14)*12</f>
+        <f t="shared" si="12"/>
         <v>8.0598378336660836E-2</v>
       </c>
     </row>
-    <row r="15" spans="2:28">
+    <row r="15" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B15" s="12">
         <v>0.15</v>
       </c>
@@ -10450,7 +10450,7 @@
         <v>23.2</v>
       </c>
       <c r="K15" s="14">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>0.39534120734908135</v>
       </c>
       <c r="L15" s="36">
@@ -10468,7 +10468,7 @@
         <v>22.58</v>
       </c>
       <c r="Q15" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>0.41437007874015747</v>
       </c>
       <c r="R15" s="36">
@@ -10479,34 +10479,34 @@
         <v>0.15</v>
       </c>
       <c r="U15" s="47">
-        <f>(E15-C15)/C15</f>
+        <f t="shared" si="7"/>
         <v>1.4749383865886014E-2</v>
       </c>
       <c r="V15" s="50">
-        <f>(K15-I15)/I15</f>
+        <f t="shared" si="8"/>
         <v>-2.2563543118791142E-2</v>
       </c>
       <c r="W15" s="50">
-        <f>(Q15-O15)/O15</f>
+        <f t="shared" si="9"/>
         <v>2.4483190905366641E-2</v>
       </c>
       <c r="Y15" s="43">
         <v>0.15</v>
       </c>
       <c r="Z15" s="12">
-        <f>(E15-C15)*12</f>
+        <f t="shared" si="10"/>
         <v>7.1587743847411289E-2</v>
       </c>
       <c r="AA15" s="53">
-        <f>(K15-I15)*12</f>
+        <f t="shared" si="11"/>
         <v>-0.10951461835731457</v>
       </c>
       <c r="AB15" s="53">
-        <f>(Q15-O15)*12</f>
+        <f t="shared" si="12"/>
         <v>0.11883183833559885</v>
       </c>
     </row>
-    <row r="16" spans="2:28">
+    <row r="16" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B16" s="12">
         <v>0.2</v>
       </c>
@@ -10536,7 +10536,7 @@
         <v>24.66</v>
       </c>
       <c r="K16" s="14">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>0.44324146981627299</v>
       </c>
       <c r="L16" s="36">
@@ -10554,7 +10554,7 @@
         <v>23.99</v>
       </c>
       <c r="Q16" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>0.46062992125984253</v>
       </c>
       <c r="R16" s="36">
@@ -10565,34 +10565,34 @@
         <v>0.2</v>
       </c>
       <c r="U16" s="47">
-        <f>(E16-C16)/C16</f>
+        <f t="shared" si="7"/>
         <v>8.5337122569809649E-3</v>
       </c>
       <c r="V16" s="50">
-        <f>(K16-I16)/I16</f>
+        <f t="shared" si="8"/>
         <v>-1.976327679195598E-2</v>
       </c>
       <c r="W16" s="50">
-        <f>(Q16-O16)/O16</f>
+        <f t="shared" si="9"/>
         <v>1.8691605761727435E-2</v>
       </c>
       <c r="Y16" s="43">
         <v>0.2</v>
       </c>
       <c r="Z16" s="12">
-        <f>(E16-C16)*12</f>
+        <f t="shared" si="10"/>
         <v>4.6305082120094321E-2</v>
       </c>
       <c r="AA16" s="53">
-        <f>(K16-I16)*12</f>
+        <f t="shared" si="11"/>
         <v>-0.10723822496652025</v>
       </c>
       <c r="AB16" s="53">
-        <f>(Q16-O16)*12</f>
+        <f t="shared" si="12"/>
         <v>0.10142319235631425</v>
       </c>
     </row>
-    <row r="17" spans="2:28">
+    <row r="17" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B17" s="12">
         <v>0.25</v>
       </c>
@@ -10622,7 +10622,7 @@
         <v>25.94</v>
       </c>
       <c r="K17" s="14">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>0.48523622047244097</v>
       </c>
       <c r="L17" s="36">
@@ -10640,7 +10640,7 @@
         <v>25.18</v>
       </c>
       <c r="Q17" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>0.49967191601049871</v>
       </c>
       <c r="R17" s="36">
@@ -10651,34 +10651,34 @@
         <v>0.25</v>
       </c>
       <c r="U17" s="47">
-        <f>(E17-C17)/C17</f>
+        <f t="shared" si="7"/>
         <v>-2.4946537886829066E-3</v>
       </c>
       <c r="V17" s="50">
-        <f>(K17-I17)/I17</f>
+        <f t="shared" si="8"/>
         <v>-1.5803597700775319E-2</v>
       </c>
       <c r="W17" s="50">
-        <f>(Q17-O17)/O17</f>
+        <f t="shared" si="9"/>
         <v>1.3476078905827697E-2</v>
       </c>
       <c r="Y17" s="43">
         <v>0.25</v>
       </c>
       <c r="Z17" s="12">
-        <f>(E17-C17)*12</f>
+        <f t="shared" si="10"/>
         <v>-1.4759205048665347E-2</v>
       </c>
       <c r="AA17" s="53">
-        <f>(K17-I17)*12</f>
+        <f t="shared" si="11"/>
         <v>-9.3499362528981056E-2</v>
       </c>
       <c r="AB17" s="53">
-        <f>(Q17-O17)*12</f>
+        <f t="shared" si="12"/>
         <v>7.9728983927711772E-2</v>
       </c>
     </row>
-    <row r="18" spans="2:28">
+    <row r="18" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B18" s="12">
         <v>0.3</v>
       </c>
@@ -10708,7 +10708,7 @@
         <v>26.96</v>
       </c>
       <c r="K18" s="14">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>0.51870078740157488</v>
       </c>
       <c r="L18" s="36">
@@ -10726,7 +10726,7 @@
         <v>26.3</v>
       </c>
       <c r="Q18" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>0.53641732283464572</v>
       </c>
       <c r="R18" s="36">
@@ -10737,34 +10737,34 @@
         <v>0.3</v>
       </c>
       <c r="U18" s="47">
-        <f>(E18-C18)/C18</f>
+        <f t="shared" si="7"/>
         <v>-4.2077667308819322E-3</v>
       </c>
       <c r="V18" s="50">
-        <f>(K18-I18)/I18</f>
+        <f t="shared" si="8"/>
         <v>-1.9708891159105894E-2</v>
       </c>
       <c r="W18" s="50">
-        <f>(Q18-O18)/O18</f>
+        <f t="shared" si="9"/>
         <v>1.3773537605858166E-2</v>
       </c>
       <c r="Y18" s="43">
         <v>0.3</v>
       </c>
       <c r="Z18" s="12">
-        <f>(E18-C18)*12</f>
+        <f t="shared" si="10"/>
         <v>-2.6717433996821249E-2</v>
       </c>
       <c r="AA18" s="53">
-        <f>(K18-I18)*12</f>
+        <f t="shared" si="11"/>
         <v>-0.12514263084721389</v>
       </c>
       <c r="AB18" s="53">
-        <f>(Q18-O18)*12</f>
+        <f t="shared" si="12"/>
         <v>8.7455794349636129E-2</v>
       </c>
     </row>
-    <row r="19" spans="2:28" ht="15.75" thickBot="1">
+    <row r="19" spans="2:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="16">
         <v>0.32</v>
       </c>
@@ -10794,7 +10794,7 @@
         <v>27.43</v>
       </c>
       <c r="K19" s="15">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>0.5341207349081365</v>
       </c>
       <c r="L19" s="37">
@@ -10812,7 +10812,7 @@
         <v>26.5</v>
       </c>
       <c r="Q19" s="15">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>0.54297900262467191</v>
       </c>
       <c r="R19" s="37">
@@ -10823,34 +10823,34 @@
         <v>0.32</v>
       </c>
       <c r="U19" s="48">
-        <f>(E19-C19)/C19</f>
+        <f t="shared" si="7"/>
         <v>-7.643020817035477E-3</v>
       </c>
       <c r="V19" s="51">
-        <f>(K19-I19)/I19</f>
+        <f t="shared" si="8"/>
         <v>-1.550447159666901E-2</v>
       </c>
       <c r="W19" s="51">
-        <f>(Q19-O19)/O19</f>
+        <f t="shared" si="9"/>
         <v>8.2315694564664684E-4</v>
       </c>
       <c r="Y19" s="44">
         <v>0.32</v>
       </c>
       <c r="Z19" s="16">
-        <f>(E19-C19)*12</f>
+        <f t="shared" si="10"/>
         <v>-4.9759038345259743E-2</v>
       </c>
       <c r="AA19" s="54">
-        <f>(K19-I19)*12</f>
+        <f t="shared" si="11"/>
         <v>-0.10094014070746482</v>
       </c>
       <c r="AB19" s="54">
-        <f>(Q19-O19)*12</f>
+        <f t="shared" si="12"/>
         <v>5.3590718909601875E-3</v>
       </c>
     </row>
-    <row r="20" spans="2:28" ht="15.75" thickBot="1">
+    <row r="20" spans="2:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
@@ -10882,7 +10882,7 @@
         <v>1.1839741572625155E-2</v>
       </c>
     </row>
-    <row r="21" spans="2:28" ht="15.75" thickBot="1">
+    <row r="21" spans="2:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E21" s="20" t="s">
         <v>13</v>
       </c>
@@ -10905,19 +10905,19 @@
         <v>1.4017948050654837E-3</v>
       </c>
     </row>
-    <row r="22" spans="2:28" ht="15.75" thickBot="1">
+    <row r="22" spans="2:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="65" t="s">
         <v>14</v>
       </c>
       <c r="C22" s="66"/>
     </row>
-    <row r="23" spans="2:28" ht="15.75" thickBot="1">
+    <row r="23" spans="2:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="63" t="s">
         <v>15</v>
       </c>
       <c r="C23" s="64"/>
     </row>
-    <row r="24" spans="2:28" ht="15.75" thickBot="1">
+    <row r="24" spans="2:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="17" t="s">
         <v>16</v>
       </c>
@@ -10925,7 +10925,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="25" spans="2:28">
+    <row r="25" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B25" s="21">
         <v>0</v>
       </c>
@@ -10934,273 +10934,273 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="2:28">
+    <row r="26" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B26" s="22">
         <v>0.02</v>
       </c>
       <c r="C26" s="25">
-        <f t="shared" ref="C26:C55" si="9">1.55*B26^2.58</f>
+        <f t="shared" ref="C26:C55" si="15">1.55*B26^2.58</f>
         <v>6.411934643775419E-5</v>
       </c>
     </row>
-    <row r="27" spans="2:28">
+    <row r="27" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B27" s="22">
         <v>0.04</v>
       </c>
       <c r="C27" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>3.8339502738176122E-4</v>
       </c>
     </row>
-    <row r="28" spans="2:28">
+    <row r="28" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B28" s="22">
         <v>0.06</v>
       </c>
       <c r="C28" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>1.0913446509460117E-3</v>
       </c>
     </row>
-    <row r="29" spans="2:28">
+    <row r="29" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B29" s="22">
         <v>0.08</v>
       </c>
       <c r="C29" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>2.2924710744479868E-3</v>
       </c>
     </row>
-    <row r="30" spans="2:28">
+    <row r="30" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B30" s="22">
         <v>0.1</v>
       </c>
       <c r="C30" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>4.0769153874378444E-3</v>
       </c>
     </row>
-    <row r="31" spans="2:28">
+    <row r="31" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B31" s="22">
         <v>0.12</v>
       </c>
       <c r="C31" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>6.525582925873622E-3</v>
       </c>
     </row>
-    <row r="32" spans="2:28">
+    <row r="32" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B32" s="22">
         <v>0.14000000000000001</v>
       </c>
       <c r="C32" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>9.7127459700171691E-3</v>
       </c>
     </row>
-    <row r="33" spans="2:3">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33" s="22">
         <v>0.16</v>
       </c>
       <c r="C33" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>1.3707594652623608E-2</v>
       </c>
     </row>
-    <row r="34" spans="2:3">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B34" s="22">
         <v>0.18</v>
       </c>
       <c r="C34" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>1.8575254011746728E-2</v>
       </c>
     </row>
-    <row r="35" spans="2:3">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B35" s="22">
         <v>0.2</v>
       </c>
       <c r="C35" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>2.4377495614638721E-2</v>
       </c>
     </row>
-    <row r="36" spans="2:3">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B36" s="22">
         <v>0.22</v>
       </c>
       <c r="C36" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>3.1173259491050275E-2</v>
       </c>
     </row>
-    <row r="37" spans="2:3">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B37" s="22">
         <v>0.24</v>
       </c>
       <c r="C37" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>3.9019050934588635E-2</v>
       </c>
     </row>
-    <row r="38" spans="2:3">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B38" s="22">
         <v>0.26</v>
       </c>
       <c r="C38" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>4.7969250841353041E-2</v>
       </c>
     </row>
-    <row r="39" spans="2:3">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B39" s="22">
         <v>0.28000000000000003</v>
       </c>
       <c r="C39" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>5.8076364061848774E-2</v>
       </c>
     </row>
-    <row r="40" spans="2:3">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B40" s="22">
         <v>0.3</v>
       </c>
       <c r="C40" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>6.9391221957620625E-2</v>
       </c>
     </row>
-    <row r="41" spans="2:3">
+    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B41" s="22">
         <v>0.32</v>
       </c>
       <c r="C41" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>8.1963150268266852E-2</v>
       </c>
     </row>
-    <row r="42" spans="2:3">
+    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B42" s="22">
         <v>0.34</v>
       </c>
       <c r="C42" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>9.5840110140021362E-2</v>
       </c>
     </row>
-    <row r="43" spans="2:3">
+    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B43" s="22">
         <v>0.36</v>
       </c>
       <c r="C43" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>0.11106881801065087</v>
       </c>
     </row>
-    <row r="44" spans="2:3">
+    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B44" s="22">
         <v>0.38</v>
       </c>
       <c r="C44" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>0.12769484857347996</v>
       </c>
     </row>
-    <row r="45" spans="2:3">
+    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B45" s="22">
         <v>0.4</v>
       </c>
       <c r="C45" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>0.14576272401257673</v>
       </c>
     </row>
-    <row r="46" spans="2:3">
+    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B46" s="22">
         <v>0.42</v>
       </c>
       <c r="C46" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>0.16531599196298566</v>
       </c>
     </row>
-    <row r="47" spans="2:3">
+    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B47" s="22">
         <v>0.44</v>
       </c>
       <c r="C47" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>0.18639729411079389</v>
       </c>
     </row>
-    <row r="48" spans="2:3">
+    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B48" s="22">
         <v>0.46</v>
       </c>
       <c r="C48" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>0.20904842694716996</v>
       </c>
     </row>
-    <row r="49" spans="2:3">
+    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B49" s="22">
         <v>0.48</v>
       </c>
       <c r="C49" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>0.23331039588807301</v>
       </c>
     </row>
-    <row r="50" spans="2:3">
+    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B50" s="22">
         <v>0.5</v>
       </c>
       <c r="C50" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>0.25922346373980926</v>
       </c>
     </row>
-    <row r="51" spans="2:3">
+    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B51" s="22">
         <v>0.52</v>
       </c>
       <c r="C51" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>0.28682719431110998</v>
       </c>
     </row>
-    <row r="52" spans="2:3">
+    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B52" s="22">
         <v>0.54</v>
       </c>
       <c r="C52" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>0.31616049183163297</v>
       </c>
     </row>
-    <row r="53" spans="2:3">
+    <row r="53" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B53" s="22">
         <v>0.56000000000000005</v>
       </c>
       <c r="C53" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>0.34726163672521515</v>
       </c>
     </row>
-    <row r="54" spans="2:3">
+    <row r="54" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B54" s="22">
         <v>0.57999999999999996</v>
       </c>
       <c r="C54" s="25">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>0.38016831819691932</v>
       </c>
     </row>
-    <row r="55" spans="2:3" ht="15.75" thickBot="1">
+    <row r="55" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B55" s="23">
         <v>0.6</v>
       </c>
       <c r="C55" s="26">
-        <f t="shared" si="9"/>
+        <f t="shared" si="15"/>
         <v>0.4149176640208378</v>
       </c>
     </row>
@@ -11221,6 +11221,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="c18885db-b23a-4ab9-857e-443224b79c26" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100675570F5CE5AA3458866B93D69FFE3C1" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d44cc85cd438149e719e50fcaa2017da">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="c18885db-b23a-4ab9-857e-443224b79c26" xmlns:ns4="1255b0f0-8c1b-44ec-8f47-a39e049da051" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f42cb373a5ea0d2e53184721f5bc8ce5" ns3:_="" ns4:_="">
     <xsd:import namespace="c18885db-b23a-4ab9-857e-443224b79c26"/>
@@ -11479,33 +11496,41 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="c18885db-b23a-4ab9-857e-443224b79c26" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F7640DE7-7DB1-41E0-BB46-687741785D9F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A641E1D-377F-4BA5-82EA-81D8C7910155}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22D68D7C-5179-4766-97DE-01476039DE5D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22D68D7C-5179-4766-97DE-01476039DE5D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c18885db-b23a-4ab9-857e-443224b79c26"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A641E1D-377F-4BA5-82EA-81D8C7910155}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F7640DE7-7DB1-41E0-BB46-687741785D9F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c18885db-b23a-4ab9-857e-443224b79c26"/>
+    <ds:schemaRef ds:uri="1255b0f0-8c1b-44ec-8f47-a39e049da051"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>